<commit_message>
fix(#126): stop None/NA strings from being converted to NaN when parsing .xlsx
Conversion of None/NA values to NaN results in those values disappearing
when the file is written back a .ags file.
</commit_message>
<xml_diff>
--- a/tests/test.xlsx
+++ b/tests/test.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="PROJ" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="150">
   <si>
     <t xml:space="preserve">HEADING</t>
   </si>
@@ -69,7 +69,10 @@
     <t xml:space="preserve">Project_Name</t>
   </si>
   <si>
-    <t xml:space="preserve">Project_Locations</t>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NA</t>
   </si>
   <si>
     <t xml:space="preserve">Contractor_Name</t>
@@ -596,7 +599,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -650,7 +653,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -660,20 +663,24 @@
       <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="D4" s="0" t="s">
+        <v>14</v>
+      </c>
       <c r="E4" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -694,34 +701,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -729,7 +736,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -740,7 +747,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
@@ -772,37 +779,37 @@
         <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -823,10 +830,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -853,7 +860,7 @@
         <v>9</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -864,7 +871,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -872,10 +879,10 @@
         <v>11</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -883,10 +890,10 @@
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -894,10 +901,10 @@
         <v>11</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -905,10 +912,10 @@
         <v>11</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -916,10 +923,10 @@
         <v>11</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -927,10 +934,10 @@
         <v>11</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -938,10 +945,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -949,10 +956,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -960,10 +967,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -971,10 +978,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -982,10 +989,10 @@
         <v>11</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -993,10 +1000,10 @@
         <v>11</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1004,10 +1011,10 @@
         <v>11</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1015,10 +1022,10 @@
         <v>11</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1026,10 +1033,10 @@
         <v>11</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1037,10 +1044,10 @@
         <v>11</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1048,16 +1055,16 @@
         <v>11</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1078,10 +1085,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1105,10 +1112,10 @@
         <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1116,10 +1123,10 @@
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1127,10 +1134,10 @@
         <v>11</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1138,10 +1145,10 @@
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1149,10 +1156,10 @@
         <v>11</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1160,10 +1167,10 @@
         <v>11</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1171,10 +1178,10 @@
         <v>11</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1182,10 +1189,10 @@
         <v>11</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1193,10 +1200,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1204,10 +1211,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1215,10 +1222,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1226,10 +1233,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1237,16 +1244,16 @@
         <v>11</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1273,46 +1280,46 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N1" s="0" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="O1" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1320,22 +1327,22 @@
         <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N2" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1346,28 +1353,28 @@
         <v>9</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>10</v>
@@ -1376,10 +1383,10 @@
         <v>10</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N3" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1387,37 +1394,37 @@
         <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>5000000.001</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K4" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="M4" s="2" t="s">
-        <v>121</v>
-      </c>
       <c r="N4" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O4" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1425,37 +1432,37 @@
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>5000000.01</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N5" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O5" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1463,37 +1470,37 @@
         <v>11</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>5000000.1</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N6" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O6" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1501,176 +1508,176 @@
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>5000000</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="N7" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O7" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F8" s="0"/>
       <c r="G8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O8" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="N10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O10" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1684,44 +1691,44 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L5"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1729,19 +1736,19 @@
         <v>7</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1758,7 +1765,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" s="0" t="s">
         <v>9</v>
@@ -1767,16 +1774,16 @@
         <v>10</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J3" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1784,31 +1791,31 @@
         <v>11</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>15.01</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H4" s="0" t="n">
         <v>15.019</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="L4" s="0" t="n">
         <v>15.1234</v>
@@ -1819,31 +1826,31 @@
         <v>11</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>15.14</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H5" s="0" t="n">
         <v>15.1432</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K5" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="L5" s="0" t="n">
         <v>15</v>
@@ -1852,7 +1859,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>